<commit_message>
fix: align delivery column names with deployed Python backend
Sheet columns renamed from domestic_delivery/international_delivery
to domestic_delivery_method/international_delivery_method to match
admin.py and generate-contract-v2.py field names.
</commit_message>
<xml_diff>
--- a/data/WCC_Contract_Data.xlsx
+++ b/data/WCC_Contract_Data.xlsx
@@ -680,7 +680,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>- domestic_delivery / international_delivery can differ for the same intake</t>
+          <t>- domestic_delivery_method / international_delivery_method can differ for the same intake</t>
         </is>
       </c>
     </row>
@@ -2261,8 +2261,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
@@ -2305,12 +2305,12 @@
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>domestic_delivery</t>
+          <t>domestic_delivery_method</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>international_delivery</t>
+          <t>international_delivery_method</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">

</xml_diff>

<commit_message>
fix: include google_drive_file_id in Outline Map tab
The Excel builder was dropping the google_drive_file_id column,
causing all programs to show hasOutline=false.
</commit_message>
<xml_diff>
--- a/data/WCC_Contract_Data.xlsx
+++ b/data/WCC_Contract_Data.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Programs'!$A$1:$D$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Intakes'!$A$1:$K$138</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Fees'!$A$1:$W$127</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Outline Map'!$A$1:$B$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Outline Map'!$A$1:$C$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -13058,11 +13058,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13076,6 +13077,11 @@
           <t>outline_filename</t>
         </is>
       </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>google_drive_file_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -13088,6 +13094,11 @@
           <t>Dementia_Care_Program_Outline</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1Bc7UIrxQyvTuAuSWhdr_KptjQIVOKUSk</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -13100,6 +13111,11 @@
           <t>Medication_Management_Program_Outline</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1MEFLML2M1qf4tUzEOT2WQ3XcryBUCbrU</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13112,6 +13128,11 @@
           <t>Palliative_Care_Program_Outline</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>17TXHg3Ez31zF_r0RV5MRqTX-ZlexcJv3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -13124,6 +13145,11 @@
           <t>Make_Up_Artistry_Fundamentals_Program_Outline</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1YhsdKwPcwkCoDpQsHVf5HWnz_uHe-ONm</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -13132,6 +13158,7 @@
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13144,6 +13171,11 @@
           <t>Canadian_Taxation_Program_Outline</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>13JBtrsK9Rpd2jxcrRCtFwD30q3IGVXk7</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -13152,6 +13184,7 @@
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -13164,6 +13197,11 @@
           <t>Keyboarding_Skills_Program_Outline</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>16mn2MMiTLi8nqRho2ShQXBYNhwKENX6w</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13176,6 +13214,11 @@
           <t>Food_Service_Assistant_Certificate_Program_Outline</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11nYt04usy7ap10IKrc2UhH-_m39l_6Oq</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13188,6 +13231,11 @@
           <t>Basics_of_Computers_Program_Outline</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>197Izf-lTwBjzSy-IVMy3P4smUQAXDhLN</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13200,6 +13248,11 @@
           <t>Network_Engineer_Program_Outline</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1Gfj6Ew2SVEA-Yi8CEaSXJGhbEQ59Zc7B</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13212,6 +13265,11 @@
           <t>Information_System_Program_Outline</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1syRGM5mpId4o2KEJiGz18UhAK81CgFjT</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13224,6 +13282,11 @@
           <t>Academic_Prep_Program_Outline</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1WqWJei6peDj7ABCYzzot5Fbi7uYExPir</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13236,6 +13299,11 @@
           <t>CLB_Test_Preparation_Program_Outline</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1y9ghwixoXnGBGlY4nPw5QLoW5_BID70V</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13248,6 +13316,11 @@
           <t>IELTS_Preparation_Program_Outline</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1gRQHCaEVHYZ6JqhVRj2pRBT2in2pwuf5</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13260,6 +13333,11 @@
           <t>Private_Pilot_License_Program_Outline</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>10EZByQPgfWic2QU3vxTj7Bs3c-S8sAqp</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13272,6 +13350,11 @@
           <t>Warehouse_and_Logistics_Fundamentals_Program_Outline</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>15-5UkT6JXUSwrlYqdsQvj7wZY3wvN41-</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13284,6 +13367,11 @@
           <t>Acute_Care_for_HCAs_Program_Outline</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1_9BNJf_UgjUMNjkzLCtlYDpCo48roXHr</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13296,6 +13384,11 @@
           <t>Accounting_Management_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>17rUFwCuBvliA8oLAKHnUfjYn4SCJ7Up8</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13308,6 +13401,11 @@
           <t>Certificate_in_Business_Essentials_Program_Outline</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1r02JVQo0whIbYtQCsYl1QQy4qy8vQEFQ</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13320,6 +13418,11 @@
           <t>Activity_Assistant_Certificate_Program_Outline</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>13o9OozmUdgok3TGSO8N3kYlN5qcdotqO</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13332,6 +13435,11 @@
           <t>Addictions_Support_Worker_Program_Outline</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1h0kd0kUaEHWW8oGVtACnlW4Rxx7XroUE</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13344,6 +13452,11 @@
           <t>Cloud_Computing_Technology_Program_Outline</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>15Enn_eFMUhU-qOTtToH2aiPHGxk_lpQm</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13356,6 +13469,11 @@
           <t>Digital_Technology_Solutions_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>16EvFsTvd2hr6BezZelVKwLC-zdGHvPEz</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13368,6 +13486,11 @@
           <t>Health_Services_Administration_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1lxqJBlpc98WqkEwf4UkEYRxL58BtG6-d</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13380,6 +13503,11 @@
           <t>Integrated_Business_Management_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1471TFOycepRTKxRQmVsngyFBjZRR4acX</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13392,6 +13520,11 @@
           <t>Network_Administrator_Program_Outline</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1Y08vVYt2Y4KSHejvGFupGPjbTbyva2gS</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13404,6 +13537,11 @@
           <t>Community_Mental_Health_Certificate_Program_Outline</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>12llLz-fdi_MSiDC5gNZrszXFydb3JjXI</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13416,6 +13554,11 @@
           <t>Commercial_Pilot_License_Program_Outline</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1hE0yzZbVsytClb4p4FYtYhw7XxitEwzq</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13428,6 +13571,11 @@
           <t>Airline_Cabin_Crew_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1Dej0N-EaQwqAg7RR9djUmWkjv_M4pWrj</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13440,6 +13588,11 @@
           <t>Gerontology_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1QU31b9cR4Lg1Frz7FFMR9WoSR0DAOHkF</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13452,6 +13605,11 @@
           <t>Flight_Instructor_Rating_Program_Outline</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1zxcdJGmKHv2OxjeNprWJKPsw5NDKqMPv</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -13464,6 +13622,11 @@
           <t>Pharmacy_Assistant_Program_Outline</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1cyk7OaYxd8oMGb_-NDWn5sbohhTSOVKC</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -13476,6 +13639,11 @@
           <t>Computer_Science_Fundamentals_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1rAqJ2Eq00ttfJFZFPiKocbPuHfY1lp0O</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -13488,6 +13656,11 @@
           <t>Network_Support_Technician_Program_Outline</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1EM1OpISsUNTbBN9pFlgAOepTwr0nVTL3</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13500,6 +13673,11 @@
           <t>HCA_Access_Program_Outline</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1b6IVqk3CYXYxkjCsh6s49iVYTWdK6yMN</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13512,6 +13690,11 @@
           <t>Medical_Office_Assistant_Program_Outline</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>10kVVqCfD4ckkIQkIWVVbMBmbuVNL7zB1</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -13524,6 +13707,11 @@
           <t>DBM_Coop_Program_Outline</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1UZvU1ZuSF87nZXxtOH0yHvUkcmpXmtTF</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -13536,6 +13724,11 @@
           <t>Dental_Receptionist_Program_Outline</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>16_YOcla93BSgR5nAlqKJa8MOFf9t_Zda</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -13548,6 +13741,11 @@
           <t>Education_Assistant_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1M5zrQ5nVaO9si-P5eSfmSO7MqGWWArs3</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -13560,6 +13758,11 @@
           <t>Office_Assistant_Certificate_Program_Outline</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>10hXJLJNK2FlnrLSZm0TFErOfpuGuL5b6</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -13572,6 +13775,11 @@
           <t>Certificate_in_International_Trade_Program_Outline</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1puDC4sGjtSX9oLwaRUEnhLMqDkqQK-3m</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -13584,6 +13792,11 @@
           <t>Hospitality_Management_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1v1Tb2Ftx6zmyvBW6JL7TD_7LtD9-Ztx9</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -13596,6 +13809,11 @@
           <t>Accounting_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1FFWkwxutjHTGam_P5DWVTAmMqFCyB6yQ</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -13608,6 +13826,11 @@
           <t>Intl_Business_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1sZsObRNvWiXT3TbmPHPqk71OcjiYZbfc</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -13620,6 +13843,11 @@
           <t>ECE_Assistant_Program_Outline</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1Cp6WRfYKbyqA3ioTN2WwAD32igmo0SGn</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -13632,6 +13860,11 @@
           <t>ESL_Program_Outline</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>16W6h6i_GQ8x09oesoBVL67bhjIEWUDfD</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -13644,6 +13877,11 @@
           <t>Medical_Device_Reprocessing_Technician_Program_Outline</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1zXVC2MbFPqIyP_BkBlQEBc_JqXfgZ8K_</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -13656,6 +13894,11 @@
           <t>Medical_Lab_Assistant_Program_Outline</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>12VkMGOLNsD27LAOws72ol73nbE3GIuL5</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -13668,6 +13911,11 @@
           <t>Night_Rating_Program_Outline</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1qvMWQlFcugUtVaTNHzwOMD4PASrNIiMW</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -13680,6 +13928,11 @@
           <t>LICG_Program_Outline</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1G9kuhzeaYMShmA8k6_wyYwesCv7Nur49</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -13692,6 +13945,11 @@
           <t>Paralegal_Studies_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1esok0CQexQGJDjtIymUvFL21AY5QWScU</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -13704,6 +13962,11 @@
           <t>Dental_Assistant_Program_Outline</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>163dmrwYuBeOL8OaDsCPDN9pAtLhgiiru</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -13716,6 +13979,11 @@
           <t>Hospitality_Management_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1v1Tb2Ftx6zmyvBW6JL7TD_7LtD9-Ztx9</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -13728,6 +13996,11 @@
           <t>Business_Management_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1gOiZAptf6pKmOv7M6uiU-VUG3XrTn2Dt</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -13740,6 +14013,11 @@
           <t>Accounting_PCP_Certificate_Program_Outline</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>1twceBoVmmFNQuhyVNMdjamqBgAxgtpAa</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -13752,6 +14030,11 @@
           <t>Bookkeeping_Accounting_Certificate_Program_Outline</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1MNa4PkcCg1lpUAlLXqQCb1WyQ36If1HH</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -13764,6 +14047,11 @@
           <t>Health_Care_Assistant_Program_Outline</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1MeL81zft6fXVsiE2pYg1gytKRoAthOhX</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -13776,6 +14064,11 @@
           <t>HCA_ESL_Program_Outline</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1IFkd9g4dt430miSNUC98AdlLM6_LDqiJ</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -13788,6 +14081,11 @@
           <t>Pharmacy_Technician_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1CLp5FMrygWOCe5tNn5vPMRXELH3wEZlw</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -13800,6 +14098,11 @@
           <t>Registered_Massage_Therapy_Program_Outline</t>
         </is>
       </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1_Xe6s2yu5hsIEVg0exZLR4UbsUbti2-3</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -13812,6 +14115,11 @@
           <t>Community_Support_Worker_Program_Outline</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1YMlFZpSMaNMHbmlcccCofufknok0dUhM</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -13824,9 +14132,14 @@
           <t>ECE_Diploma_Program_Outline</t>
         </is>
       </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1LgxY5-otD3pyxN-gHn9999Q6h4N63wWD</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B64"/>
+  <autoFilter ref="A1:C64"/>
   <conditionalFormatting sqref="A2:A200">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>ISBLANK(A2)</formula>

</xml_diff>